<commit_message>
Fix seven Basic UDI criteria to FALSE (sync engine, simplify UI form)
Sync eudamed_tool workbook/importer from Eudamed-Upload: implantable,
reusable, administering_medicine and the tissue/substance criteria are
pinned to false and no longer workbook columns (legacy columns ignored).
Basic UDI form now shows only Active device and Measuring function; the
pinned criteria are noted as fixed. XML output still contains all
elements (XSD-required), always false.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/eudamed_master_data.xlsx
+++ b/templates/eudamed_master_data.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -437,15 +437,8 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="22" customWidth="1" min="7" max="7"/>
-    <col width="21" customWidth="1" min="8" max="8"/>
-    <col width="21" customWidth="1" min="9" max="9"/>
-    <col width="25" customWidth="1" min="10" max="10"/>
-    <col width="24" customWidth="1" min="11" max="11"/>
-    <col width="14" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
-    <col width="14" customWidth="1" min="15" max="15"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -481,52 +474,17 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>animal_tissues_cells</t>
+          <t>active</t>
         </is>
       </c>
       <c r="H1" s="2" t="inlineStr">
         <is>
-          <t>human_tissues_cells</t>
-        </is>
-      </c>
-      <c r="I1" s="2" t="inlineStr">
-        <is>
-          <t>human_product_check</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>medicinal_product_check</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>administering_medicine</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>active</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>implantable</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
           <t>measuring_function</t>
-        </is>
-      </c>
-      <c r="O1" s="2" t="inlineStr">
-        <is>
-          <t>reusable</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="12">
+  <dataValidations count="5">
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"EUDAMED,GS1,HIBCC,ICCBBA,IFA"</formula1>
     </dataValidation>
@@ -540,27 +498,6 @@
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
     <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="L2:L201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M2:M201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="N2:N201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="O2:O201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Fix device flags/reuses/base quantity, reduce PI selection (sync + UI)
Sync eudamed_tool from Eudamed-Upload. Device form no longer shows the
five flags, number of reuses or base quantity - all fixed portfolio
values (false / -1 / 1) noted in the form. Production identifier
choices reduced to SERIALISATION_NUMBER, MANUFACTURING_DATE,
SOFTWARE_IDENTIFICATION.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/eudamed_master_data.xlsx
+++ b/templates/eudamed_master_data.xlsx
@@ -511,7 +511,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O1"/>
+  <dimension ref="A1:H1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -519,16 +519,9 @@
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="18" customWidth="1" min="4" max="4"/>
     <col width="15" customWidth="1" min="5" max="5"/>
-    <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="15" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="15" customWidth="1" min="9" max="9"/>
-    <col width="14" customWidth="1" min="10" max="10"/>
-    <col width="14" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="14" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="19" customWidth="1" min="15" max="15"/>
+    <col width="18" customWidth="1" min="6" max="6"/>
+    <col width="18" customWidth="1" min="7" max="7"/>
+    <col width="19" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -559,77 +552,27 @@
       </c>
       <c r="F1" s="2" t="inlineStr">
         <is>
-          <t>sterile</t>
+          <t>intended_purpose</t>
         </is>
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
-          <t>sterilization</t>
-        </is>
-      </c>
-      <c r="H1" s="1" t="inlineStr">
-        <is>
-          <t>number_of_reuses</t>
-        </is>
-      </c>
-      <c r="I1" s="1" t="inlineStr">
-        <is>
-          <t>base_quantity</t>
-        </is>
-      </c>
-      <c r="J1" s="2" t="inlineStr">
-        <is>
-          <t>latex</t>
-        </is>
-      </c>
-      <c r="K1" s="2" t="inlineStr">
-        <is>
-          <t>reprocessed</t>
-        </is>
-      </c>
-      <c r="L1" s="2" t="inlineStr">
-        <is>
-          <t>intended_purpose</t>
-        </is>
-      </c>
-      <c r="M1" s="2" t="inlineStr">
-        <is>
-          <t>single_use</t>
-        </is>
-      </c>
-      <c r="N1" s="2" t="inlineStr">
-        <is>
           <t>software_version</t>
         </is>
       </c>
-      <c r="O1" s="2" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>direct_marking_di</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="7">
+  <dataValidations count="2">
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"EUDAMED,GS1,HIBCC,ICCBBA,IFA"</formula1>
     </dataValidation>
     <dataValidation sqref="E2:E201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"ON_THE_MARKET,NOT_INTENDED_FOR_EU_MARKET,NO_LONGER_PLACED_ON_THE_MARKET"</formula1>
-    </dataValidation>
-    <dataValidation sqref="F2:F201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="G2:G201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="K2:K201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
-    </dataValidation>
-    <dataValidation sqref="M2:M201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
-      <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -742,7 +685,7 @@
   </sheetData>
   <dataValidations count="1">
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
-      <formula1>"BATCH_NUMBER,SERIALISATION_NUMBER,MANUFACTURING_DATE,EXPIRATION_DATE,SOFTWARE_IDENTIFICATION"</formula1>
+      <formula1>"SERIALISATION_NUMBER,MANUFACTURING_DATE,SOFTWARE_IDENTIFICATION"</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Add specialDevice + VAL-015 software / SOFTWARE_IDENTIFICATION coupling
specialDevice (MDRSpecialDeviceTypeEnum) added to the Basic UDI-DI model, ORM (migration e5f6a7b8c9d0), converter, workbook and Basic UDI form; emitted in the generated XML. VAL-015 (error) enforces EUDAMED's rule coupling a software specialDevice (e.g. MDR_SOFTWARE) with the SOFTWARE_IDENTIFICATION production identifier. Demo monitor marked MDR_SOFTWARE.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/eudamed_master_data.xlsx
+++ b/templates/eudamed_master_data.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H1"/>
+  <dimension ref="A1:I1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -437,8 +437,9 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="14" customWidth="1" min="7" max="7"/>
-    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="16" customWidth="1" min="7" max="7"/>
+    <col width="14" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -474,17 +475,22 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>special_device</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>active</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>measuring_function</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"EUDAMED,GS1,HIBCC,ICCBBA,IFA"</formula1>
     </dataValidation>
@@ -495,9 +501,12 @@
       <formula1>"DEVICE,SYSTEM,PROCEDURE_PACK"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"MDR_SOFTWARE,MDR_STANDARD_SOFT_CONTACT_LENSES,MDR_RIGID_GAS_PERMEABLE,MDR_MADE_TO_ORDER,MDR_SPECTACLES_FRAMES,MDR_SPECTACLES_LENSES,MDR_READY_MADE_SPECTACLES,MDR_ORTHOPEDIC,MDR_MADE_TO_ORDER_RIGID_GAS_PERMEABLE,MDD_SOFTWARE,MDD_STANDARD_SOFT_CONTACT_LENSES,MDD_RIGID_GAS_PERMEABLE,MDD_MADE_TO_ORDER,MDD_SPECTACLES_FRAMES,MDD_SPECTACLES_LENSES,MDD_READY_MADE_SPECTACLES,MDD_ORTHOPEDIC,AIMDD_SOFTWARE,AIMDD_ORTHOPEDIC"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>

<commit_message>
Add Legacy device (MDD/AIMDD) submission support
applicable_legislation on Basic UDI-DI (MDR/MDD/AIMDD) with ORM column (migration f6a7b8c9d0e1), converter, workbook and form. Legacy -> device:Device xsi:type=MDEUDeviceType (MDEUData+MDEUDI, eudi:applicableLegislation) on DEVICE.POST; additional UDI-DIs xsi:type=eudididata:MDEUDataType on UDI_DI.POST. XSD-validated.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/templates/eudamed_master_data.xlsx
+++ b/templates/eudamed_master_data.xlsx
@@ -428,7 +428,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I1"/>
+  <dimension ref="A1:J1"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -437,9 +437,10 @@
     <col width="14" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="24" customWidth="1" min="7" max="7"/>
+    <col width="16" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -475,22 +476,27 @@
       </c>
       <c r="G1" s="2" t="inlineStr">
         <is>
+          <t>applicable_legislation</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
+        <is>
           <t>special_device</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>active</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>measuring_function</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <dataValidations count="6">
+  <dataValidations count="7">
     <dataValidation sqref="B2:B201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" type="list">
       <formula1>"EUDAMED,GS1,HIBCC,ICCBBA,IFA"</formula1>
     </dataValidation>
@@ -501,12 +507,15 @@
       <formula1>"DEVICE,SYSTEM,PROCEDURE_PACK"</formula1>
     </dataValidation>
     <dataValidation sqref="G2:G201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+      <formula1>"MDR,MDD,AIMDD"</formula1>
+    </dataValidation>
+    <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"MDR_SOFTWARE,MDR_STANDARD_SOFT_CONTACT_LENSES,MDR_RIGID_GAS_PERMEABLE,MDR_MADE_TO_ORDER,MDR_SPECTACLES_FRAMES,MDR_SPECTACLES_LENSES,MDR_READY_MADE_SPECTACLES,MDR_ORTHOPEDIC,MDR_MADE_TO_ORDER_RIGID_GAS_PERMEABLE,MDD_SOFTWARE,MDD_STANDARD_SOFT_CONTACT_LENSES,MDD_RIGID_GAS_PERMEABLE,MDD_MADE_TO_ORDER,MDD_SPECTACLES_FRAMES,MDD_SPECTACLES_LENSES,MDD_READY_MADE_SPECTACLES,MDD_ORTHOPEDIC,AIMDD_SOFTWARE,AIMDD_ORTHOPEDIC"</formula1>
     </dataValidation>
-    <dataValidation sqref="H2:H201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
-    <dataValidation sqref="I2:I201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
+    <dataValidation sqref="J2:J201" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" type="list">
       <formula1>"TRUE,FALSE"</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>